<commit_message>
research(agent-sandbox): 샌드박스 내부 해부 신규 글 + ZDR/HIPAA 설명 보강
## 신규 글 — 에이전트 샌드박스 내부 해부
앞 글 6장이 "왜/어디에"(경계)를 다뤘다면, 이 글은 "어떻게"(구현 층위)를 다룬다.

- 1장 격리 단위: 기술 경계 4층(컨테이너 → gVisor → microVM → isolate/WASM)과
  논리 단위(세션당·툴 호출당·컨테이너 객체당·액터당)를 분리
- 2장 구현 언어: Firecracker=Rust, gVisor=Go — 격리 장치가 뚫리면 격리가 무의미하므로
  메모리 안전성이 곧 보안 요구사항. 벤더별 채택 현황
- 3장 실행 언어: Python(결과물이 목적) vs TypeScript(오케스트레이션이 목적)의 상이한 근거
- 4장 동시성: 테넌트 격리 / 세션 어피니티·스코프 키 / 콜드스타트 세 문제로 분해
- 5장 로컬 샌드박스: Claude Code의 Seatbelt·bubblewrap·WFP, 서버와 다른 위협 모델

Mermaid 3개(엣지 애니메이션 fast), 퀴즈 7문항, 참고문헌 17건에 [N] 인라인 인용.
1차 자료 우선, 벤더 비교 자료는 2차 출처로 명시.
Mermaid 3/3 렌더링·에러 0 검증 완료.

## 기존 글 보강
8.1절에 ZDR/HIPAA BAA 설명 콜아웃 추가. Anthropic 기능별 적격성 표로
"compaction은 ZDR 유지 가능 / Managed Agents·code execution은 비적격" 주장을 확인.
참고문헌 [55] 추가 (블로그·XLSX 동시).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2026-09-15-model-agent-api-session-memory/model-agent-api-session-memory-references.xlsx
+++ b/2026-09-15-model-agent-api-session-memory/model-agent-api-session-memory-references.xlsx
@@ -11,7 +11,7 @@
     <sheet name="상태소유권_매트릭스" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'참고문헌'!$A$1:$G$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'참고문헌'!$A$1:$G$56</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -93,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -135,6 +135,12 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -508,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -571,12 +577,12 @@
           <t>OpenAI 공식 문서</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="15" t="inlineStr">
         <is>
           <t>https://developers.openai.com/api/docs/guides/conversation-state</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E2" s="16" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -586,7 +592,7 @@
           <t>대화 상태 관리 4가지 방식 정리: 수동 메시지 전달, previous_response_id 체이닝, Conversations API, store 파라미터. 체인의 모든 이전 입력 토큰이 입력 토큰으로 과금된다는 점과 응답 30일 보존, Conversation 객체는 30일 TTL 미적용이라는 점이 핵심.</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G2" s="16" t="inlineStr">
         <is>
           <t>3.1, 2</t>
         </is>
@@ -606,12 +612,12 @@
           <t>OpenAI 공식 문서</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="13" t="inlineStr">
         <is>
           <t>https://developers.openai.com/api/docs/guides/migrate-to-responses</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E3" s="14" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -621,7 +627,7 @@
           <t>Chat Completions는 대화 상태를 직접 관리해야 하지만 Responses API는 Conversations API 연동 또는 previous_response_id로 상태를 서버가 관리. Chat Completions는 계속 지원되어 흐름 단위 점진 이전 가능.</t>
         </is>
       </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="G3" s="14" t="inlineStr">
         <is>
           <t>3.1</t>
         </is>
@@ -641,12 +647,12 @@
           <t>OpenAI Agents SDK 문서</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>https://openai.github.io/openai-agents-python/sessions/</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="16" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -656,7 +662,7 @@
           <t>세션 구현체 목록: MemorySession(프로세스 메모리), SQLiteSession(기본 인메모리·경로 지정 시 영속), OpenAIConversationsSession(OpenAI 서버 동기화), OpenAIResponsesCompactionSession(자동 압축), Redis/SQLAlchemy/MongoDB/Dapr.</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="16" t="inlineStr">
         <is>
           <t>4.3, 6</t>
         </is>
@@ -676,12 +682,12 @@
           <t>OpenAI Agents SDK 문서</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>https://openai.github.io/openai-agents-python/models/</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="14" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -691,7 +697,7 @@
           <t>LiteLLM 및 Any-LLM 어댑터를 통해 비 OpenAI 모델 사용 가능(베스트에포트 베타). OpenAI 모델과 타 벤더 모델을 혼합하는 시나리오용.</t>
         </is>
       </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="G5" s="14" t="inlineStr">
         <is>
           <t>4.3, 6</t>
         </is>
@@ -711,12 +717,12 @@
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="15" t="inlineStr">
         <is>
           <t>https://openai.com/index/introducing-agentkit/</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="16" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
@@ -726,7 +732,7 @@
           <t>AgentKit = Agents SDK + Responses API + ChatKit + Agent Builder 번들. 공통 과금·API 표면을 공유.</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G6" s="16" t="inlineStr">
         <is>
           <t>4.3</t>
         </is>
@@ -746,12 +752,12 @@
           <t>OpenAI 공식 문서</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="13" t="inlineStr">
         <is>
           <t>https://developers.openai.com/api/docs/guides/chatkit</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E7" s="14" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -761,7 +767,7 @@
           <t>Agent Builder는 2026-11-30 종료 예정이며 ChatKit은 영향 없음. 신규 작업은 ChatKit SDK + Agents SDK 기반 자체 서버 구현 권장. 셀프호스팅 옵션 제공.</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
+      <c r="G7" s="14" t="inlineStr">
         <is>
           <t>4.3</t>
         </is>
@@ -781,12 +787,12 @@
           <t>Anthropic 공식 문서</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="15" t="inlineStr">
         <is>
           <t>https://platform.claude.com/docs/en/managed-agents/overview</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="16" t="inlineStr">
         <is>
           <t>2026-04</t>
         </is>
@@ -796,7 +802,7 @@
           <t>Agent/Environment/Session/Events 4개 개념. 이벤트 이력은 서버에 영속되고 전체 조회 가능. 베타 헤더 managed-agents-2026-04-01. 설계상 상태 저장이라 ZDR·HIPAA BAA 적용 대상이 아님.</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G8" s="16" t="inlineStr">
         <is>
           <t>4.1, 5, 7.1</t>
         </is>
@@ -816,12 +822,12 @@
           <t>Anthropic 공식 문서</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>https://platform.claude.com/docs/en/managed-agents/sessions</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -831,7 +837,7 @@
           <t>POST /v1/sessions (agent, environment_id 필수), POST /v1/sessions/{id}/events. initial_events 최대 50개. agent 오버라이드는 병합이 아닌 전체 치환. budget.max_list_cost는 센트 단위 문자열. vault_ids로 MCP OAuth 위임.</t>
         </is>
       </c>
-      <c r="G9" s="9" t="inlineStr">
+      <c r="G9" s="14" t="inlineStr">
         <is>
           <t>4.1</t>
         </is>
@@ -851,12 +857,12 @@
           <t>Anthropic 공식 문서</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="15" t="inlineStr">
         <is>
           <t>https://platform.claude.com/docs/en/managed-agents/memory</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="16" t="inlineStr">
         <is>
           <t>2026-07</t>
         </is>
@@ -866,7 +872,7 @@
           <t>베타 헤더 agent-memory-2026-07-22. /v1/memory_stores. 세션 resources[]로 부착 후 /mnt/memory/&lt;slug&gt;/에 마운트. 세션당 8개, 메모리당 100kB, store당 1만 개. 불변 memory version + redact. read_write 기본값의 프롬프트 인젝션 위험 경고.</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G10" s="16" t="inlineStr">
         <is>
           <t>4.1, 6</t>
         </is>
@@ -886,12 +892,12 @@
           <t>Anthropic 공식 문서</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D11" s="13" t="inlineStr">
         <is>
           <t>https://platform.claude.com/docs/en/build-with-claude/context-editing</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="E11" s="14" t="inlineStr">
         <is>
           <t>2025-2026</t>
         </is>
@@ -901,7 +907,7 @@
           <t>베타 헤더 context-management-2025-06-27. clear_tool_uses_20250919 전략으로 오래된 tool result를 시간순 제거하고 자리표시 텍스트로 대체. applied_edits로 제거량 보고.</t>
         </is>
       </c>
-      <c r="G11" s="9" t="inlineStr">
+      <c r="G11" s="14" t="inlineStr">
         <is>
           <t>3.2</t>
         </is>
@@ -921,12 +927,12 @@
           <t>Anthropic 공식 문서</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="15" t="inlineStr">
         <is>
           <t>https://platform.claude.com/docs/en/build-with-claude/compaction</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E12" s="16" t="inlineStr">
         <is>
           <t>2026-01</t>
         </is>
@@ -936,7 +942,7 @@
           <t>베타 헤더 compact-2026-01-12, 전략 compact_20260112. 트리거 기본 input_tokens 150,000(최소 50,000). 클라이언트가 여전히 전체 메시지 목록을 전송하고 API가 compaction 블록 이전을 드롭. pause_after_compaction, instructions 지원.</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G12" s="16" t="inlineStr">
         <is>
           <t>3.2, 7.2</t>
         </is>
@@ -956,12 +962,12 @@
           <t>Anthropic 공식 문서</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="D13" s="13" t="inlineStr">
         <is>
           <t>https://platform.claude.com/docs/en/agents-and-tools/tool-use/memory-tool</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="E13" s="14" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
@@ -971,7 +977,7 @@
           <t>memory_20250818 클라이언트 사이드 메모리 툴. 에이전트가 툴 호출을 하면 애플리케이션이 로컬에서 실행하므로 저장 위치와 방식을 개발자가 통제.</t>
         </is>
       </c>
-      <c r="G13" s="9" t="inlineStr">
+      <c r="G13" s="14" t="inlineStr">
         <is>
           <t>3.2</t>
         </is>
@@ -991,12 +997,12 @@
           <t>Anthropic / Claude Code 문서</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="15" t="inlineStr">
         <is>
           <t>https://code.claude.com/docs/en/agent-sdk/sessions</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="16" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -1006,7 +1012,7 @@
           <t>세션은 ~/.claude/projects/ 아래 프로젝트 경로 해시 디렉터리에 .jsonl(append-only)로 저장. ID로 resume, fork 시 새 session ID로 분기.</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G14" s="16" t="inlineStr">
         <is>
           <t>4.2</t>
         </is>
@@ -1026,12 +1032,12 @@
           <t>Anthropic 블로그</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>https://claude.com/blog/claude-managed-agents-updates</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="E15" s="14" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -1041,7 +1047,7 @@
           <t>self-hosted 샌드박스에서는 툴 실행만 자체 인프라로 이동하고 오케스트레이션·컨텍스트 관리·오류 복구는 Anthropic 인프라에 잔류. MCP 터널로 사내망 MCP 서버를 아웃바운드 연결만으로 노출.</t>
         </is>
       </c>
-      <c r="G15" s="9" t="inlineStr">
+      <c r="G15" s="14" t="inlineStr">
         <is>
           <t>4.1, 7.1</t>
         </is>
@@ -1061,12 +1067,12 @@
           <t>Google AI for Developers</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="15" t="inlineStr">
         <is>
           <t>https://ai.google.dev/gemini-api/docs/interactions-overview</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E16" s="16" t="inlineStr">
         <is>
           <t>2026-06</t>
         </is>
@@ -1076,7 +1082,7 @@
           <t>2026-06 GA. previous_interaction_id로 서버 상태 체이닝, store 기본 true. 보존 유료 55일(7/14/28 조정)·무료 1일. tools/system_instruction/generation_config는 interaction 스코프라 승계되지 않음.</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="G16" s="16" t="inlineStr">
         <is>
           <t>3.3</t>
         </is>
@@ -1096,12 +1102,12 @@
           <t>Google AI for Developers</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
+      <c r="D17" s="13" t="inlineStr">
         <is>
           <t>https://ai.google.dev/gemini-api/docs/interactions</t>
         </is>
       </c>
-      <c r="E17" s="9" t="inlineStr">
+      <c r="E17" s="14" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -1111,7 +1117,7 @@
           <t>무상태 요청-응답 모델. 클라이언트가 전체 대화 이력을 배열로 유지해야 함.</t>
         </is>
       </c>
-      <c r="G17" s="9" t="inlineStr">
+      <c r="G17" s="14" t="inlineStr">
         <is>
           <t>3.3</t>
         </is>
@@ -1131,12 +1137,12 @@
           <t>Google AI for Developers</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D18" s="15" t="inlineStr">
         <is>
           <t>https://ai.google.dev/gemini-api/docs/caching</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E18" s="16" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -1146,7 +1152,7 @@
           <t>Gemini 2.5 이후 implicit caching 기본 활성. 상태(previous_interaction_id) 모드와 무상태 모드 모두 지원.</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="G18" s="16" t="inlineStr">
         <is>
           <t>3.3, 7.2</t>
         </is>
@@ -1166,12 +1172,12 @@
           <t>Google Cloud 문서</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
+      <c r="D19" s="13" t="inlineStr">
         <is>
           <t>https://cloud.google.com/agent-builder/agent-engine/memory-bank/overview</t>
         </is>
       </c>
-      <c r="E19" s="9" t="inlineStr">
+      <c r="E19" s="14" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -1181,7 +1187,7 @@
           <t>사용자-에이전트 대화에서 기억을 저장하는 동적 시스템. 세션을 넘어 과거 대화 데이터를 참조해 개인화 응답 제공.</t>
         </is>
       </c>
-      <c r="G19" s="9" t="inlineStr">
+      <c r="G19" s="14" t="inlineStr">
         <is>
           <t>4.6</t>
         </is>
@@ -1201,12 +1207,12 @@
           <t>Google Cloud 문서</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D20" s="15" t="inlineStr">
         <is>
           <t>https://cloud.google.com/vertex-ai/generative-ai/docs/agent-engine/memory-bank/generate-memories</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E20" s="16" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -1216,7 +1222,7 @@
           <t>GenerateMemories로 세션/턴 종료 시점에 사실 자동 추출, RetrieveMemories로 전체 조회 또는 유사도 검색 조회. scope 딕셔너리(예: session_id)로 범위 지정, 같은 스코프끼리만 통합. 미지정 시 user_id로 자동 키잉.</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="G20" s="16" t="inlineStr">
         <is>
           <t>4.6</t>
         </is>
@@ -1236,12 +1242,12 @@
           <t>Google Cloud 블로그</t>
         </is>
       </c>
-      <c r="D21" s="8" t="inlineStr">
+      <c r="D21" s="13" t="inlineStr">
         <is>
           <t>https://cloud.google.com/blog/products/ai-machine-learning/vertex-ai-memory-bank-in-public-preview</t>
         </is>
       </c>
-      <c r="E21" s="9" t="inlineStr">
+      <c r="E21" s="14" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
@@ -1251,7 +1257,7 @@
           <t>Memory Bank 최초 공개. ADK 및 Agent Engine Sessions와 통합.</t>
         </is>
       </c>
-      <c r="G21" s="9" t="inlineStr">
+      <c r="G21" s="14" t="inlineStr">
         <is>
           <t>4.6</t>
         </is>
@@ -1271,12 +1277,12 @@
           <t>Google Cloud 문서</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D22" s="15" t="inlineStr">
         <is>
           <t>https://docs.cloud.google.com/agent-builder/agent-engine/memory-bank/quickstart-api</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E22" s="16" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -1286,7 +1292,7 @@
           <t>Agent Engine SDK는 프레임워크 오케스트레이션 없이도, ADK가 아닌 프레임워크와도 Sessions·Memory Bank 사용 가능. REST API 직접 호출 경로 문서화.</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="G22" s="16" t="inlineStr">
         <is>
           <t>4.6, 6</t>
         </is>
@@ -1306,12 +1312,12 @@
           <t>Google Cloud 문서</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
+      <c r="D23" s="13" t="inlineStr">
         <is>
           <t>https://docs.cloud.google.com/vertex-ai/generative-ai/docs/release-notes</t>
         </is>
       </c>
-      <c r="E23" s="9" t="inlineStr">
+      <c r="E23" s="14" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -1321,7 +1327,7 @@
           <t>Agent Engine Sessions·Memory Bank GA. 2026-01-28부터 Sessions·Memory Bank·Code Execution 과금 시작.</t>
         </is>
       </c>
-      <c r="G23" s="9" t="inlineStr">
+      <c r="G23" s="14" t="inlineStr">
         <is>
           <t>4.6</t>
         </is>
@@ -1341,12 +1347,12 @@
           <t>AWS 공식 문서</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D24" s="15" t="inlineStr">
         <is>
           <t>https://docs.aws.amazon.com/bedrock-agentcore/latest/devguide/memory.html</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="E24" s="16" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -1356,7 +1362,7 @@
           <t>완전관리형 메모리 서비스. 단기(세션 내 turn-by-turn)와 장기(세션 간 선호·사실·요약) 구분. 다양한 SDK·에이전트 프레임워크 지원.</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr">
+      <c r="G24" s="16" t="inlineStr">
         <is>
           <t>4.4</t>
         </is>
@@ -1376,12 +1382,12 @@
           <t>AWS 공식 문서</t>
         </is>
       </c>
-      <c r="D25" s="8" t="inlineStr">
+      <c r="D25" s="13" t="inlineStr">
         <is>
           <t>https://docs.aws.amazon.com/bedrock-agentcore/latest/devguide/memory-terminology.html</t>
         </is>
       </c>
-      <c r="E25" s="9" t="inlineStr">
+      <c r="E25" s="14" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -1391,7 +1397,7 @@
           <t>Memory(최상위 컨테이너), Strategy(단기→장기 변환 규칙), Namespace(구조화된 경로), Memory record(구조화 단위), Session(sessionId), Actor(actorId), Event(CreateEvent로 저장, 불변·타임스탬프).</t>
         </is>
       </c>
-      <c r="G25" s="9" t="inlineStr">
+      <c r="G25" s="14" t="inlineStr">
         <is>
           <t>4.4</t>
         </is>
@@ -1411,12 +1417,12 @@
           <t>AWS 공식 문서</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D26" s="15" t="inlineStr">
         <is>
           <t>https://docs.aws.amazon.com/bedrock-agentcore/latest/devguide/using-memory-short-term.html</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E26" s="16" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -1426,7 +1432,7 @@
           <t>단기: CreateEvent/GetEvent/ListEvents/DeleteEvent. 장기: 전략 설정 후 RetrieveMemoryRecords/ListMemoryRecords/DeleteMemoryRecords, 네임스페이스 조직, 구조화 메타데이터, 실패 재처리(redrive).</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
+      <c r="G26" s="16" t="inlineStr">
         <is>
           <t>4.4</t>
         </is>
@@ -1446,12 +1452,12 @@
           <t>AWS What's New</t>
         </is>
       </c>
-      <c r="D27" s="8" t="inlineStr">
+      <c r="D27" s="13" t="inlineStr">
         <is>
           <t>https://aws.amazon.com/about-aws/whats-new/2026/09/agentcore-memory-direct-ingest/</t>
         </is>
       </c>
-      <c r="E27" s="9" t="inlineStr">
+      <c r="E27" s="14" t="inlineStr">
         <is>
           <t>2026-09</t>
         </is>
@@ -1461,7 +1467,7 @@
           <t>IngestData API. 콘텐츠를 받아 장기 메모리 전략들로 팬아웃하고 단기 이벤트를 만들지 않고 바로 장기 레코드 생성. 대화가 아닌 문서를 메모리에 넣는 경로.</t>
         </is>
       </c>
-      <c r="G27" s="9" t="inlineStr">
+      <c r="G27" s="14" t="inlineStr">
         <is>
           <t>4.4</t>
         </is>
@@ -1481,12 +1487,12 @@
           <t>AWS What's New</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D28" s="15" t="inlineStr">
         <is>
           <t>https://aws.amazon.com/about-aws/whats-new/2026/03/agentcore-memory-streaming-ltm</t>
         </is>
       </c>
-      <c r="E28" s="5" t="inlineStr">
+      <c r="E28" s="16" t="inlineStr">
         <is>
           <t>2026-03</t>
         </is>
@@ -1496,7 +1502,7 @@
           <t>장기 메모리 레코드 생성·변경 시 푸시 알림. 폴링 불필요.</t>
         </is>
       </c>
-      <c r="G28" s="5" t="inlineStr">
+      <c r="G28" s="16" t="inlineStr">
         <is>
           <t>4.4</t>
         </is>
@@ -1516,12 +1522,12 @@
           <t>AWS What's New</t>
         </is>
       </c>
-      <c r="D29" s="8" t="inlineStr">
+      <c r="D29" s="13" t="inlineStr">
         <is>
           <t>https://aws.amazon.com/about-aws/whats-new/2026/05/agentcore-memory-scmetadata/</t>
         </is>
       </c>
-      <c r="E29" s="9" t="inlineStr">
+      <c r="E29" s="14" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -1531,7 +1537,7 @@
           <t>애플리케이션이 붙인 메타데이터가 LLM 추론 없이 추출·통합을 그대로 통과해 장기 레코드에 도달.</t>
         </is>
       </c>
-      <c r="G29" s="9" t="inlineStr">
+      <c r="G29" s="14" t="inlineStr">
         <is>
           <t>4.4</t>
         </is>
@@ -1551,12 +1557,12 @@
           <t>AWS 공식 문서</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D30" s="15" t="inlineStr">
         <is>
           <t>https://docs.aws.amazon.com/bedrock-agentcore/latest/devguide/runtime-sessions.html</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr">
+      <c r="E30" s="16" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -1566,7 +1572,7 @@
           <t>세션마다 전용 microVM(컴퓨트·메모리·파일시스템 격리). 세션 헤더로 동일 microVM 라우팅, 클라이언트가 세션 ID를 이후 요청에 포함해야 어피니티 유지. 최대 8시간, 15분 무활동 시 회수.</t>
         </is>
       </c>
-      <c r="G30" s="5" t="inlineStr">
+      <c r="G30" s="16" t="inlineStr">
         <is>
           <t>4.4</t>
         </is>
@@ -1586,12 +1592,12 @@
           <t>AWS What's New</t>
         </is>
       </c>
-      <c r="D31" s="8" t="inlineStr">
+      <c r="D31" s="13" t="inlineStr">
         <is>
           <t>https://aws.amazon.com/about-aws/whats-new/2026/03/bedrock-agentcore-runtime-session-storage</t>
         </is>
       </c>
-      <c r="E31" s="9" t="inlineStr">
+      <c r="E31" s="14" t="inlineStr">
         <is>
           <t>2026-03</t>
         </is>
@@ -1601,7 +1607,7 @@
           <t>에이전트 파일시스템 상태를 유지하는 관리형 세션 스토리지 프리뷰.</t>
         </is>
       </c>
-      <c r="G31" s="9" t="inlineStr">
+      <c r="G31" s="14" t="inlineStr">
         <is>
           <t>4.4</t>
         </is>
@@ -1621,12 +1627,12 @@
           <t>AWS 블로그</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D32" s="15" t="inlineStr">
         <is>
           <t>https://aws.amazon.com/blogs/machine-learning/evaluate-any-agent-framework-with-amazon-bedrock-agentcore-evaluations/</t>
         </is>
       </c>
-      <c r="E32" s="5" t="inlineStr">
+      <c r="E32" s="16" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -1636,7 +1642,7 @@
           <t>AgentCore Runtime은 프레임워크 무관이며 Bedrock·Anthropic Claude·Google Gemini·OpenAI 등 서로 다른 LLM으로 실행 가능. OTel 텔레메트리만 있으면 평가도 프레임워크 무관.</t>
         </is>
       </c>
-      <c r="G32" s="5" t="inlineStr">
+      <c r="G32" s="16" t="inlineStr">
         <is>
           <t>4.4, 6</t>
         </is>
@@ -1656,12 +1662,12 @@
           <t>AWS 공식 문서</t>
         </is>
       </c>
-      <c r="D33" s="8" t="inlineStr">
+      <c r="D33" s="13" t="inlineStr">
         <is>
           <t>https://docs.aws.amazon.com/bedrock/latest/userguide/sessions.html</t>
         </is>
       </c>
-      <c r="E33" s="9" t="inlineStr">
+      <c r="E33" s="14" t="inlineStr">
         <is>
           <t>2025-2026</t>
         </is>
@@ -1671,7 +1677,7 @@
           <t>CreateSession → CreateInvocation → PutInvocationStep. 세밀한 상태 체크포인트(텍스트·이미지) 저장. 자동 주입형이 아닌 명시적 저장형.</t>
         </is>
       </c>
-      <c r="G33" s="9" t="inlineStr">
+      <c r="G33" s="14" t="inlineStr">
         <is>
           <t>3.5, 6</t>
         </is>
@@ -1691,12 +1697,12 @@
           <t>AWS 블로그</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="D34" s="15" t="inlineStr">
         <is>
           <t>https://aws.amazon.com/blogs/machine-learning/amazon-bedrock-launches-session-management-apis-for-generative-ai-applications-preview/</t>
         </is>
       </c>
-      <c r="E34" s="5" t="inlineStr">
+      <c r="E34" s="16" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
@@ -1706,7 +1712,7 @@
           <t>LangGraph·LlamaIndex 등 오픈소스 프레임워크의 상태·컨텍스트 관리 단순화를 목적으로 설계.</t>
         </is>
       </c>
-      <c r="G34" s="5" t="inlineStr">
+      <c r="G34" s="16" t="inlineStr">
         <is>
           <t>3.5, 6</t>
         </is>
@@ -1726,12 +1732,12 @@
           <t>hidekazu-konishi.com</t>
         </is>
       </c>
-      <c r="D35" s="8" t="inlineStr">
+      <c r="D35" s="13" t="inlineStr">
         <is>
           <t>https://hidekazu-konishi.com/entry/amazon_bedrock_converse_api_deep_dive.html</t>
         </is>
       </c>
-      <c r="E35" s="9" t="inlineStr">
+      <c r="E35" s="14" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
@@ -1741,7 +1747,7 @@
           <t>Converse는 무상태로, 호출자가 messages 배열을 관리하고 매 요청 전체 이력을 재전송해야 하며 Bedrock은 이를 보관하지 않음. InvokeAgent는 반대로 sessionId 기반 서버 세션.</t>
         </is>
       </c>
-      <c r="G35" s="9" t="inlineStr">
+      <c r="G35" s="14" t="inlineStr">
         <is>
           <t>3.5</t>
         </is>
@@ -1761,12 +1767,12 @@
           <t>Microsoft Learn</t>
         </is>
       </c>
-      <c r="D36" s="4" t="inlineStr">
+      <c r="D36" s="15" t="inlineStr">
         <is>
           <t>https://learn.microsoft.com/en-us/azure/ai-foundry/agents/concepts/threads-runs-messages</t>
         </is>
       </c>
-      <c r="E36" s="5" t="inlineStr">
+      <c r="E36" s="16" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -1776,7 +1782,7 @@
           <t>스레드는 명시적 삭제 전까지 유지되고 최대 10만 메시지 부착 가능. Standard setup에서는 고객 Azure Cosmos DB에 저장. Run은 스레드에 대해 에이전트를 기동하는 단위.</t>
         </is>
       </c>
-      <c r="G36" s="5" t="inlineStr">
+      <c r="G36" s="16" t="inlineStr">
         <is>
           <t>4.5</t>
         </is>
@@ -1796,12 +1802,12 @@
           <t>Microsoft Learn</t>
         </is>
       </c>
-      <c r="D37" s="8" t="inlineStr">
+      <c r="D37" s="13" t="inlineStr">
         <is>
           <t>https://learn.microsoft.com/en-us/azure/foundry/openai/how-to/responses</t>
         </is>
       </c>
-      <c r="E37" s="9" t="inlineStr">
+      <c r="E37" s="14" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -1811,7 +1817,7 @@
           <t>previous_response_id로 새 메시지만 전송하고 서비스가 이력을 이어붙임. 대화 상태 30일 유지(또는 삭제 시까지).</t>
         </is>
       </c>
-      <c r="G37" s="9" t="inlineStr">
+      <c r="G37" s="14" t="inlineStr">
         <is>
           <t>3.4</t>
         </is>
@@ -1831,12 +1837,12 @@
           <t>Azure Cosmos DB 블로그</t>
         </is>
       </c>
-      <c r="D38" s="4" t="inlineStr">
+      <c r="D38" s="15" t="inlineStr">
         <is>
           <t>https://devblogs.microsoft.com/cosmosdb/azure-ai-foundry-connection-for-azure-cosmos-db-and-byo-thread-storage-in-azure-ai-agent-service/</t>
         </is>
       </c>
-      <c r="E38" s="5" t="inlineStr">
+      <c r="E38" s="16" t="inlineStr">
         <is>
           <t>2025-2026</t>
         </is>
@@ -1846,7 +1852,7 @@
           <t>enterprise_memory DB 안에 thread-message-store(사용자 대화), system-thread-message-store(내부 시스템 메시지), agent-entity-store(모델 입출력) 컨테이너 생성. 고객 계정에 저장.</t>
         </is>
       </c>
-      <c r="G38" s="5" t="inlineStr">
+      <c r="G38" s="16" t="inlineStr">
         <is>
           <t>4.5, 7.1</t>
         </is>
@@ -1866,12 +1872,12 @@
           <t>Microsoft Learn</t>
         </is>
       </c>
-      <c r="D39" s="8" t="inlineStr">
+      <c r="D39" s="13" t="inlineStr">
         <is>
           <t>https://learn.microsoft.com/en-us/azure/foundry/agents/concepts/standard-agent-setup</t>
         </is>
       </c>
-      <c r="E39" s="9" t="inlineStr">
+      <c r="E39" s="14" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -1881,7 +1887,7 @@
           <t>Standard setup은 고객 관리·단일 테넌트 리소스에 모든 고객 데이터를 저장. Cosmos DB 계정은 총 처리량 한도 3,000 RU/s 이상 필요.</t>
         </is>
       </c>
-      <c r="G39" s="9" t="inlineStr">
+      <c r="G39" s="14" t="inlineStr">
         <is>
           <t>4.5, 7.1</t>
         </is>
@@ -1901,12 +1907,12 @@
           <t>Microsoft Learn</t>
         </is>
       </c>
-      <c r="D40" s="4" t="inlineStr">
+      <c r="D40" s="15" t="inlineStr">
         <is>
           <t>https://learn.microsoft.com/en-us/azure/foundry/responsible-ai/openai/data-privacy</t>
         </is>
       </c>
-      <c r="E40" s="5" t="inlineStr">
+      <c r="E40" s="16" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -1916,7 +1922,7 @@
           <t>Responses API 등 상태 저장 엔티티 관련 데이터는 고객 Azure 테넌트의 Foundry 리소스 내부, 해당 리소스와 같은 지리에 저장되고 기본 AES-256 암호화.</t>
         </is>
       </c>
-      <c r="G40" s="5" t="inlineStr">
+      <c r="G40" s="16" t="inlineStr">
         <is>
           <t>3.4, 7.1</t>
         </is>
@@ -1936,12 +1942,12 @@
           <t>Microsoft Learn</t>
         </is>
       </c>
-      <c r="D41" s="8" t="inlineStr">
+      <c r="D41" s="13" t="inlineStr">
         <is>
           <t>https://learn.microsoft.com/en-us/azure/foundry/agents/overview</t>
         </is>
       </c>
-      <c r="E41" s="9" t="inlineStr">
+      <c r="E41" s="14" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -1951,7 +1957,7 @@
           <t>non-OpenAI 모델 지원 및 Azure AI Search·Bing Grounding·Azure Functions 등 툴 통합.</t>
         </is>
       </c>
-      <c r="G41" s="9" t="inlineStr">
+      <c r="G41" s="14" t="inlineStr">
         <is>
           <t>4.5</t>
         </is>
@@ -1971,12 +1977,12 @@
           <t>Mem0 블로그</t>
         </is>
       </c>
-      <c r="D42" s="4" t="inlineStr">
+      <c r="D42" s="15" t="inlineStr">
         <is>
           <t>https://mem0.ai/blog/mem0-vs-zep</t>
         </is>
       </c>
-      <c r="E42" s="5" t="inlineStr">
+      <c r="E42" s="16" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -1986,7 +1992,7 @@
           <t>mem0는 서비스 무관 범용 메모리 API(add/update/delete/retrieve)로 어떤 오케스트레이터 뒤에도 배치 가능. OpenMemory MCP라는 로컬 우선 메모리 서버 보유.</t>
         </is>
       </c>
-      <c r="G42" s="5" t="inlineStr">
+      <c r="G42" s="16" t="inlineStr">
         <is>
           <t>4.7</t>
         </is>
@@ -2006,12 +2012,12 @@
           <t>DEV Community</t>
         </is>
       </c>
-      <c r="D43" s="8" t="inlineStr">
+      <c r="D43" s="13" t="inlineStr">
         <is>
           <t>https://dev.to/plur9/mem0-vs-letta-vs-zep-which-should-you-use-for-agent-memory-1n8m</t>
         </is>
       </c>
-      <c r="E43" s="9" t="inlineStr">
+      <c r="E43" s="14" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -2021,7 +2027,7 @@
           <t>Zep은 Graphiti 엔진 기반 시간 인식 지식 그래프(사실의 학습 시점과 관계 보존, 공식 MCP 서버), Letta는 OS식 계층 메모리를 에이전트가 직접 편집하는 상태 저장 에이전트 OS. 셋 다 Apache-2.0, MCP 연동 방식은 상이.</t>
         </is>
       </c>
-      <c r="G43" s="9" t="inlineStr">
+      <c r="G43" s="14" t="inlineStr">
         <is>
           <t>4.7</t>
         </is>
@@ -2041,12 +2047,12 @@
           <t>Packer et al., arXiv:2310.08560</t>
         </is>
       </c>
-      <c r="D44" s="4" t="inlineStr">
+      <c r="D44" s="15" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2310.08560</t>
         </is>
       </c>
-      <c r="E44" s="5" t="inlineStr">
+      <c r="E44" s="16" t="inlineStr">
         <is>
           <t>2023-10</t>
         </is>
@@ -2056,7 +2062,7 @@
           <t>Letta의 전신. OS 가상 메모리 개념을 차용해 제한된 컨텍스트 윈도를 계층적으로 관리하는 아이디어를 제시. 현대 에이전트 메모리 제품군의 이론적 출발점.</t>
         </is>
       </c>
-      <c r="G44" s="5" t="inlineStr">
+      <c r="G44" s="16" t="inlineStr">
         <is>
           <t>4.7</t>
         </is>
@@ -2076,12 +2082,12 @@
           <t>Leonie Monigatti</t>
         </is>
       </c>
-      <c r="D45" s="8" t="inlineStr">
+      <c r="D45" s="13" t="inlineStr">
         <is>
           <t>https://www.leoniemonigatti.com/blog/claude-memory-tool.html</t>
         </is>
       </c>
-      <c r="E45" s="9" t="inlineStr">
+      <c r="E45" s="14" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
@@ -2091,7 +2097,7 @@
           <t>Anthropic 메모리 툴이 클라이언트 사이드로 동작한다는 점과 context editing과의 조합을 실습 관점에서 정리.</t>
         </is>
       </c>
-      <c r="G45" s="9" t="inlineStr">
+      <c r="G45" s="14" t="inlineStr">
         <is>
           <t>3.2</t>
         </is>
@@ -2111,12 +2117,12 @@
           <t>Matteo Bracco, Data Reply IT (Medium)</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
+      <c r="D46" s="15" t="inlineStr">
         <is>
           <t>https://medium.com/data-reply-it-datatech/stateful-agents-on-amazon-bedrock-how-agentcore-runtime-solves-the-memory-problem-74ba885776e7</t>
         </is>
       </c>
-      <c r="E46" s="5" t="inlineStr">
+      <c r="E46" s="16" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -2126,7 +2132,7 @@
           <t>AgentCore Runtime의 세션 격리와 상태 관리를 실무 관점에서 해설. 2026-02 Stateful Runtime Environment 발표 맥락 포함.</t>
         </is>
       </c>
-      <c r="G46" s="5" t="inlineStr">
+      <c r="G46" s="16" t="inlineStr">
         <is>
           <t>4.4</t>
         </is>
@@ -2146,12 +2152,12 @@
           <t>Goran Minov, Google Cloud Community (Medium)</t>
         </is>
       </c>
-      <c r="D47" s="8" t="inlineStr">
+      <c r="D47" s="13" t="inlineStr">
         <is>
           <t>https://medium.com/google-cloud/architecting-stateful-agents-with-the-gemini-interactions-api-279b195c0818</t>
         </is>
       </c>
-      <c r="E47" s="9" t="inlineStr">
+      <c r="E47" s="14" t="inlineStr">
         <is>
           <t>2026-07</t>
         </is>
@@ -2161,7 +2167,7 @@
           <t>generateContent의 무상태 한계와 Interactions API의 상태 모델 전환을 아키텍처 관점에서 비교.</t>
         </is>
       </c>
-      <c r="G47" s="9" t="inlineStr">
+      <c r="G47" s="14" t="inlineStr">
         <is>
           <t>3.3</t>
         </is>
@@ -2181,12 +2187,12 @@
           <t>Sean Goedecke</t>
         </is>
       </c>
-      <c r="D48" s="4" t="inlineStr">
+      <c r="D48" s="15" t="inlineStr">
         <is>
           <t>https://www.seangoedecke.com/responses-api/</t>
         </is>
       </c>
-      <c r="E48" s="5" t="inlineStr">
+      <c r="E48" s="16" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
@@ -2196,7 +2202,7 @@
           <t>Responses API가 전체 대화 대신 상태 ID를 주고받는 구조라는 점과 그 설계 의도에 대한 비평적 해설.</t>
         </is>
       </c>
-      <c r="G48" s="5" t="inlineStr">
+      <c r="G48" s="16" t="inlineStr">
         <is>
           <t>3.1</t>
         </is>
@@ -2447,8 +2453,43 @@
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>API and data retention (ZDR·HIPAA readiness)</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>Anthropic 공식 문서</t>
+        </is>
+      </c>
+      <c r="D56" s="17" t="inlineStr">
+        <is>
+          <t>https://platform.claude.com/docs/en/manage-claude/api-and-data-retention</t>
+        </is>
+      </c>
+      <c r="E56" s="18" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>ZDR은 응답 반환 후 프롬프트·응답을 저장하지 않는 조직 단위 계약. Managed Agents는 stateful 리소스라 비적격. HIPAA readiness는 BAA 체결 후 PHI 처리용이며 즉시 삭제 대신 암호화·접근통제·감사 로깅을 적용. 기능별 적격성 표에서 context editing·compaction·memory tool은 ZDR 적격, Managed Agents·code execution은 비적격.</t>
+        </is>
+      </c>
+      <c r="G56" s="18" t="inlineStr">
+        <is>
+          <t>8.1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G55"/>
+  <autoFilter ref="A1:G56"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -2504,6 +2545,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId55"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>